<commit_message>
Write report Section 4 (Task 3) and finalise for submission
Fill Section 4 from Riccardo's committed Task 3 results (40-token pipeline):
development table (RNN -> LSTM -> larger LSTM -> Word2Vec, validation), final
test table (EN->IT 7.26, IT->EN 9.60, character 3.86 BLEU), the into-English vs
into-Italian and word vs character comparisons, and the sentence-length analysis
with a figure. All numbers verified against results/task3_outputs.

Also: add the headline result to the abstract, fill the Task 3 rows of the Excel
sheet, and set \DRAFTfalse so the draft notes no longer print.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ExperimentSummarySheet_Ex1.xlsx
+++ b/ExperimentSummarySheet_Ex1.xlsx
@@ -52,7 +52,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +67,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -89,7 +94,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -107,6 +112,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -870,149 +878,173 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Vasilis &amp; Riccardo</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>RNN seq2seq (vanilla encoder-decoder) [Riccardo]</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>word-level, learned emb</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Task 2: lowercase, whitespace-normalised, empty/XML pairs removed; kept punctuation/numbers/stopwords</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>70/10/20, seed 42; &lt;=20 tokens</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>see Task 3 notebook</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr"/>
-      <c r="I8" s="6" t="inlineStr"/>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>Collapsed to a generic 'la &lt;unk&gt;' output</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="inlineStr">
-        <is>
-          <t>PRE-FIX DATA - RICCARDO TO UPDATE after clean re-run</t>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>word, learned emb</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Task 2 clean text; 40-token cap; regex tokenizer; 20k vocab on train</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>70/10/20, seed 42 (110,265 / 15,751 / 31,503)</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>emb 64, hidden 128</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>1.89</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>13.19</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>Weak: generic output; motivates switching to LSTM</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>validation (dev) scores</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Vasilis &amp; Riccardo</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>LSTM seq2seq, context-fed [Riccardo]</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>word-level; random vs Word2Vec emb</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Task 2: lowercase, whitespace-normalised, empty/XML pairs removed; kept punctuation/numbers/stopwords</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>70/10/20, seed 42; &lt;=20 tokens</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>hidden 128/256 tuned on val</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr"/>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>Word2Vec best on validation</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>PRE-FIX DATA - RICCARDO TO UPDATE (his committed EN-&gt;IT test was BLEU 4.20 / METEOR 19.41 on quoted data)</t>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>LSTM seq2seq + Word2Vec (best) [Riccardo]</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>word, Word2Vec-init emb</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Task 2 clean text; 40-token cap; regex tokenizer; 20k vocab on train</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>70/10/20, seed 42 (110,265 / 15,751 / 31,503)</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>emb 128, hidden 512, lr 1e-3, batch 128, Adam, grad-clip, early stopping, greedy decode</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>7.26</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>28.12</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>EN-&gt;IT test. IT-&gt;EN test = 9.60 / 33.94 (into-English is easier)</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>final selected model</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Vasilis &amp; Riccardo</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>+ IT-&gt;EN direction / character-based model [Riccardo]</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>word vs character</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Task 2: lowercase, whitespace-normalised, empty/XML pairs removed; kept punctuation/numbers/stopwords</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>70/10/20, seed 42; &lt;=20 tokens</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr"/>
-      <c r="I10" s="6" t="inlineStr"/>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
-          <t>RICCARDO - remaining Task 3 sub-tasks</t>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Character-based LSTM [Riccardo]</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>character</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Task 2 clean text; 40-token cap; regex tokenizer; 20k vocab on train</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>70/10/20, seed 42 (110,265 / 15,751 / 31,503)</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>emb 128, hidden 512, lr 1e-3, batch 128, Adam, grad-clip, early stopping, greedy decode</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>3.86</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>19.83</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>EN-&gt;IT test; worse than word model despite no OOV (longer sequences)</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>representation comparison</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel: update Task 4 rows to aligned run (7.32->18.41, emb128/hid512/20ep, <=40 split)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ExperimentSummarySheet_Ex1.xlsx
+++ b/ExperimentSummarySheet_Ex1.xlsx
@@ -562,106 +562,114 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Vasilis &amp; Riccardo</t>
+          <t xml:space="preserve">Vasilis &amp; Riccardo</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>LSTM seq2seq encoder-decoder (no attention)</t>
+          <t xml:space="preserve">LSTM seq2seq encoder-decoder (no attention)</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>word-level, learned emb (64)</t>
+          <t xml:space="preserve">word-level, Word2Vec-init emb (128)</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Task 2: lowercase, whitespace-normalised, empty/XML pairs removed; kept punctuation/numbers/stopwords</t>
+          <t xml:space="preserve">Task 2: lowercase, whitespace-normalised, empty/XML pairs removed; kept punctuation/numbers/stopwords; regex tokenizer</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>70/10/20, seed 42; &lt;=20 tokens (49,641 train)</t>
+          <t xml:space="preserve">70/10/20, seed 42; &lt;=40 tokens (110,265 / 15,751 / 31,503)</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>emb 64, hidden 256, lr 1e-3, batch 128, 12 epochs, Adam, grad-clip 1.0, greedy decode, best-val checkpoint</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="n">
-        <v>4.16</v>
-      </c>
-      <c r="I2" s="5" t="n">
-        <v>18.76</v>
+          <t xml:space="preserve">emb 128, hidden 512, lr 1e-3, batch 128, 20 epochs, Adam, grad-clip 1.0, greedy decode, best-val checkpoint (best epoch 7)</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7.32</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28.01</t>
+        </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Fixed single context vector is the bottleneck; generic outputs; quality falls with sentence length</t>
+          <t xml:space="preserve">Fixed single context vector is the bottleneck; generic outputs; quality falls with sentence length</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Retrained here as the with/without-attention baseline (same seed &amp; data)</t>
+          <t xml:space="preserve">Retrained here as the with/without-attention baseline (same seed &amp; data); ~52.8 min on Colab T4</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Vasilis &amp; Riccardo</t>
+          <t xml:space="preserve">Vasilis &amp; Riccardo</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>LSTM seq2seq + Bahdanau (additive) attention</t>
+          <t xml:space="preserve">LSTM seq2seq + Bahdanau (additive) attention</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>word-level, learned emb (64)</t>
+          <t xml:space="preserve">word-level, Word2Vec-init emb (128)</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Task 2: lowercase, whitespace-normalised, empty/XML pairs removed; kept punctuation/numbers/stopwords</t>
+          <t xml:space="preserve">Task 2: lowercase, whitespace-normalised, empty/XML pairs removed; kept punctuation/numbers/stopwords; regex tokenizer</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>70/10/20, seed 42; &lt;=20 tokens (49,641 train)</t>
+          <t xml:space="preserve">70/10/20, seed 42; &lt;=40 tokens (110,265 / 15,751 / 31,503)</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>emb 64, hidden 256, lr 1e-3, batch 128, 12 epochs, Adam, grad-clip 1.0, greedy decode, best-val checkpoint; attention masked over padding (best epoch 8)</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="n">
-        <v>7.68</v>
-      </c>
-      <c r="I3" s="5" t="n">
-        <v>27.07</v>
+          <t xml:space="preserve">emb 128, hidden 512, lr 1e-3, batch 128, 20 epochs, Adam, grad-clip 1.0, greedy decode, best-val checkpoint; attention masked over padding (best epoch 4)</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18.41</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43.69</t>
+        </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>+85% BLEU vs baseline; gain grows with length (+13% at 1-4 tok -&gt; +148% at 15-20); learns monotonic alignment</t>
+          <t xml:space="preserve">+152% BLEU vs baseline; gain grows with length (+7.0 BLEU at 1-10 tok -&gt; +11.6 at 21-30); learns monotonic alignment</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>Colab T4, ~8 min both models. Heatmap in results/task4_outputs</t>
+          <t xml:space="preserve">Colab T4, ~166 min (attention) vs ~53 min (baseline). Heatmap in results/task4_outputs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Task 5: write Pivot section and update Excel rows with aligned run
Pivot 12.04 BLEU ~= direct 12.13; oracle 19.19 shows 7.15 BLEU lost to
leg-1 error propagation; 131,225 triples, emb128/hid512/20ep.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ExperimentSummarySheet_Ex1.xlsx
+++ b/ExperimentSummarySheet_Ex1.xlsx
@@ -676,212 +676,228 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Vasilis &amp; Riccardo</t>
+          <t xml:space="preserve">Vasilis &amp; Riccardo</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>IT-&gt;EN  (pivot leg 1) LSTM+attention</t>
+          <t xml:space="preserve">IT-&gt;EN  (pivot leg 1) LSTM+attention</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>word-level, learned emb (64)</t>
+          <t xml:space="preserve">word-level, Word2Vec-init emb (128)</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>IT-EN-SV triples: join it-en &amp; sv-en on shared English side</t>
+          <t xml:space="preserve">IT-EN-SV triples: join it-en &amp; sv-en on shared English side; Task 3 pipeline (regex tokenizer, 20k vocab)</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>70/10/20 of 59,524 triples (41,668 train)</t>
+          <t xml:space="preserve">70/10/20 of 131,225 triples (91,858 / 13,122 / 26,245)</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>emb 64, hidden 256, lr 1e-3, batch 128, 12 epochs, Adam, grad-clip 1.0, greedy decode, best-val checkpoint</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>10.68</v>
-      </c>
-      <c r="I4" s="5" t="n">
-        <v>32.23</v>
+          <t xml:space="preserve">emb 128, hidden 512, lr 1e-3, batch 128, 20 epochs, Word2Vec-init, Adam, grad-clip 1.0, greedy decode, best-val checkpoint (best epoch 5)</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21.61</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">49.00</t>
+        </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Strongest of the three systems</t>
+          <t xml:space="preserve">Strongest of the four systems; leg-1 quality caps the pivot</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>Same architecture as Task 4</t>
+          <t xml:space="preserve">Same architecture as Task 4; ~132 min on Colab T4</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Vasilis &amp; Riccardo</t>
+          <t xml:space="preserve">Vasilis &amp; Riccardo</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>EN-&gt;SV  (pivot leg 2, ORACLE input) LSTM+attention</t>
+          <t xml:space="preserve">EN-&gt;SV  (pivot leg 2, ORACLE input) LSTM+attention</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>word-level, learned emb (64)</t>
+          <t xml:space="preserve">word-level, Word2Vec-init emb (128)</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>as above</t>
+          <t xml:space="preserve">as above</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>as above (41,668 train)</t>
+          <t xml:space="preserve">as above</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>emb 64, hidden 256, lr 1e-3, batch 128, 12 epochs, Adam, grad-clip 1.0, greedy decode, best-val checkpoint</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="I5" s="5" t="n">
-        <v>35.12</v>
+          <t xml:space="preserve">emb 128, hidden 512, lr 1e-3, batch 128, 20 epochs, Word2Vec-init, Adam, grad-clip 1.0, greedy decode, best-val checkpoint (best epoch 4)</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">19.19</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">48.18</t>
+        </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Evaluated on REFERENCE English -&gt; leg-2 ceiling</t>
+          <t xml:space="preserve">Evaluated on REFERENCE English -&gt; leg-2 ceiling (oracle)</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>Shares its model with the pivot row; difference = inherited error</t>
+          <t xml:space="preserve">Shares its model with the pivot row; difference = inherited error</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Vasilis &amp; Riccardo</t>
+          <t xml:space="preserve">Vasilis &amp; Riccardo</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>IT-&gt;EN-&gt;SV  (PIVOT) LSTM+attention</t>
+          <t xml:space="preserve">IT-&gt;EN-&gt;SV  (PIVOT) LSTM+attention</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>word-level, learned emb (64)</t>
+          <t xml:space="preserve">word-level, Word2Vec-init emb (128)</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>as above</t>
+          <t xml:space="preserve">as above</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>test = 11,904 triples</t>
+          <t xml:space="preserve">test = 26,245 triples</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>emb 64, hidden 256, lr 1e-3, batch 128, 12 epochs, Adam, grad-clip 1.0, greedy decode, best-val checkpoint</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>5.95</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>22.86</v>
+          <t xml:space="preserve">emb 128, hidden 512, lr 1e-3, batch 128, 20 epochs, Word2Vec-init, Adam, grad-clip 1.0, greedy decode, best-val checkpoint</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12.04</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">36.30</t>
+        </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Retains only 54% of the oracle; 5.05 BLEU lost to leg-1 errors (quality multiplicative along the chain)</t>
+          <t xml:space="preserve">Retains 62.7% of the oracle; 7.15 BLEU lost to leg-1 errors (error propagation)</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>Leg 2 fed leg 1's OWN output (no reference leak)</t>
+          <t xml:space="preserve">Leg 2 fed leg 1's OWN output (no reference leak)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Vasilis &amp; Riccardo</t>
+          <t xml:space="preserve">Vasilis &amp; Riccardo</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>IT-&gt;SV  (DIRECT, comparison) LSTM+attention</t>
+          <t xml:space="preserve">IT-&gt;SV  (DIRECT, comparison) LSTM+attention</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>word-level, learned emb (64)</t>
+          <t xml:space="preserve">word-level, Word2Vec-init emb (128)</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>as above</t>
+          <t xml:space="preserve">as above</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>test = 11,904 triples</t>
+          <t xml:space="preserve">test = 26,245 triples</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>emb 64, hidden 256, lr 1e-3, batch 128, 12 epochs, Adam, grad-clip 1.0, greedy decode, best-val checkpoint</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>6.06</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>25.08</v>
+          <t xml:space="preserve">emb 128, hidden 512, lr 1e-3, batch 128, 20 epochs, Word2Vec-init, Adam, grad-clip 1.0, greedy decode, best-val checkpoint (best epoch 4)</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12.13</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38.06</t>
+        </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>~= pivot on BLEU (gap 0.11); METEOR +2.22 over pivot; weak ceiling (same 41,668 triples)</t>
+          <t xml:space="preserve">~= pivot on BLEU (gap 0.09); METEOR +1.76 over pivot; both limited by the same data</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>Upper bound the pivot targets</t>
+          <t xml:space="preserve">Upper bound the pivot targets; ~124 min</t>
         </is>
       </c>
     </row>

</xml_diff>